<commit_message>
docs: record completed P0 roadmap milestones
</commit_message>
<xml_diff>
--- a/planning_cast_semgrep_comparator.xlsx
+++ b/planning_cast_semgrep_comparator.xlsx
@@ -1337,7 +1337,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
+    <row r="17" ht="70" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
           <t>S3.2</t>
@@ -1386,7 +1386,8 @@
       <c r="L17" s="4" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Une référence sourcée est une preuve issue des contenus éditeur; elle reste distincte de toute inférence ou opinion.</t>
+          <t>Une référence sourcée est une preuve issue des contenus éditeur; elle reste distincte de toute inférence ou opinion.
+Avancement 26/10/2026 : 6 517 candidats calculés, tous classés comme propositions indéterminées avant revue.</t>
         </is>
       </c>
     </row>
@@ -1940,14 +1941,14 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>En cours</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr"/>
       <c r="L28" s="4" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>Avancement 26/10/2026 : Code et données locales opérationnels ; publication du dépôt en cours.</t>
+          <t>Avancement 26/10/2026 : Code et données locales opérationnels ; publication sur GitHub main réalisée.</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2129,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Les P0 réalisés sont indiqués « Terminé » dans Roadmap. Les archives CAST et Semgrep restent locales. M4 passe à « Terminé » après publication effective du dépôt.</t>
+          <t>Les P0 sont indiqués « Terminé » dans Roadmap. 2 828 règles CAST authentifiées et 2 153 règles Semgrep sont importées ; 6 517 paires candidates sont calculées. Archives et base restent locales. Le code et le planning sont publiés sur GitHub main.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: refine sourced matching and multi-category exploration
</commit_message>
<xml_diff>
--- a/planning_cast_semgrep_comparator.xlsx
+++ b/planning_cast_semgrep_comparator.xlsx
@@ -1387,7 +1387,7 @@
       <c r="M17" s="2" t="inlineStr">
         <is>
           <t>Une référence sourcée est une preuve issue des contenus éditeur; elle reste distincte de toute inférence ou opinion.
-Avancement 26/10/2026 : 6 517 candidats calculés, tous classés comme propositions indéterminées avant revue.</t>
+Avancement 26/10/2026 : 4 516 candidats calculés, tous classés comme propositions indéterminées avant revue.</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Les P0 sont indiqués « Terminé » dans Roadmap. 2 828 règles CAST authentifiées et 2 153 règles Semgrep sont importées ; 6 517 paires candidates sont calculées. Archives et base restent locales. Le code et le planning sont publiés sur GitHub main.</t>
+          <t>Les P0 sont indiqués « Terminé » dans Roadmap. 2 828 règles CAST authentifiées et 2 153 règles Semgrep sont importées ; 4 516 paires candidates sont calculées. Archives et base restent locales. Le code et le planning sont publiés sur GitHub main.</t>
         </is>
       </c>
     </row>

</xml_diff>